<commit_message>
data: Clackamas 2021 covariates, thermal sensitivity metrics, and data dictionary
</commit_message>
<xml_diff>
--- a/clackamas_thermal_sensitivity_covariates_2021.xlsx
+++ b/clackamas_thermal_sensitivity_covariates_2021.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\savan\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6B8E1C1-3239-443C-8DDD-A55B5670B8B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FF29836-0AD5-4F88-A81B-D2D2653C673C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -817,7 +817,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -827,6 +827,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF494949"/>
+        <bgColor rgb="FF494949"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF155289"/>
+        <bgColor rgb="FF494949"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF3436A2"/>
         <bgColor rgb="FF494949"/>
       </patternFill>
     </fill>
@@ -843,20 +855,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -864,6 +879,12 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF3436A2"/>
+      <color rgb="FF155289"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -11456,58 +11477,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N1" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="O1" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="P1" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="Q1" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="R1" s="5" t="s">
         <v>160</v>
       </c>
     </row>
@@ -15560,870 +15581,870 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="6" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="4" t="s">
+      <c r="A2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>250</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>254</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="37.799999999999997" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>248</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>249</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="37.799999999999997" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="37.799999999999997" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="3" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="3" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="3" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="3" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="3" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="37.799999999999997" x14ac:dyDescent="0.3">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="3" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="3" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="3" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="3" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="3" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="3" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="3" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="3" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D25" s="3" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A26" s="4" t="s">
+      <c r="A26" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="C26" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D26" s="3" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A27" s="4" t="s">
+      <c r="A27" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="C27" s="4" t="s">
+      <c r="C27" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D27" s="3" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A28" s="4" t="s">
+      <c r="A28" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="B28" s="3" t="s">
         <v>208</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D28" s="3" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A29" s="4" t="s">
+      <c r="A29" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="B29" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="C29" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="D29" s="4" t="s">
+      <c r="D29" s="3" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A30" s="4" t="s">
+      <c r="A30" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="B30" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="C30" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="D30" s="4" t="s">
+      <c r="D30" s="3" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A31" s="4" t="s">
+      <c r="A31" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B31" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="C31" s="4" t="s">
+      <c r="C31" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="D31" s="4" t="s">
+      <c r="D31" s="3" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A32" s="4" t="s">
+      <c r="A32" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="B32" s="3" t="s">
         <v>213</v>
       </c>
-      <c r="C32" s="4" t="s">
+      <c r="C32" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="D32" s="4" t="s">
+      <c r="D32" s="3" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33" s="4" t="s">
+      <c r="A33" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B33" s="4" t="s">
+      <c r="B33" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="C33" s="4" t="s">
+      <c r="C33" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="D33" s="4" t="s">
+      <c r="D33" s="3" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A34" s="4" t="s">
+      <c r="A34" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="B34" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="C34" s="4" t="s">
+      <c r="C34" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="D34" s="4" t="s">
+      <c r="D34" s="3" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35" s="4" t="s">
+      <c r="A35" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B35" s="4" t="s">
+      <c r="B35" s="3" t="s">
         <v>217</v>
       </c>
-      <c r="C35" s="4" t="s">
+      <c r="C35" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="D35" s="4" t="s">
+      <c r="D35" s="3" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A36" s="4" t="s">
+      <c r="A36" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B36" s="4" t="s">
+      <c r="B36" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="C36" s="4" t="s">
+      <c r="C36" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="D36" s="4" t="s">
+      <c r="D36" s="3" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A37" s="4" t="s">
+      <c r="A37" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B37" s="4" t="s">
+      <c r="B37" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="C37" s="4" t="s">
+      <c r="C37" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="D37" s="4" t="s">
+      <c r="D37" s="3" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A38" s="4" t="s">
+      <c r="A38" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B38" s="4" t="s">
+      <c r="B38" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="C38" s="4" t="s">
+      <c r="C38" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="D38" s="4" t="s">
+      <c r="D38" s="3" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A39" s="4" t="s">
+      <c r="A39" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B39" s="4" t="s">
+      <c r="B39" s="3" t="s">
         <v>221</v>
       </c>
-      <c r="C39" s="4" t="s">
+      <c r="C39" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="D39" s="4" t="s">
+      <c r="D39" s="3" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A40" s="4" t="s">
+      <c r="A40" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B40" s="4" t="s">
+      <c r="B40" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="C40" s="4" t="s">
+      <c r="C40" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="D40" s="4" t="s">
+      <c r="D40" s="3" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A41" s="4" t="s">
+      <c r="A41" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B41" s="4" t="s">
+      <c r="B41" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="C41" s="4" t="s">
+      <c r="C41" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="D41" s="4" t="s">
+      <c r="D41" s="3" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A42" s="4" t="s">
+      <c r="A42" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B42" s="4" t="s">
+      <c r="B42" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="C42" s="4" t="s">
+      <c r="C42" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="D42" s="4" t="s">
+      <c r="D42" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A43" s="4" t="s">
+      <c r="A43" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B43" s="4" t="s">
+      <c r="B43" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="C43" s="4" t="s">
+      <c r="C43" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="D43" s="4" t="s">
+      <c r="D43" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A44" s="4" t="s">
+      <c r="A44" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B44" s="4" t="s">
+      <c r="B44" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="C44" s="4" t="s">
+      <c r="C44" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="D44" s="4" t="s">
+      <c r="D44" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A45" s="4" t="s">
+      <c r="A45" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B45" s="4" t="s">
+      <c r="B45" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="C45" s="4" t="s">
+      <c r="C45" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="D45" s="4" t="s">
+      <c r="D45" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A46" s="4" t="s">
+      <c r="A46" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B46" s="4" t="s">
+      <c r="B46" s="3" t="s">
         <v>229</v>
       </c>
-      <c r="C46" s="4" t="s">
+      <c r="C46" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="D46" s="4" t="s">
+      <c r="D46" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A47" s="4" t="s">
+      <c r="A47" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B47" s="4" t="s">
+      <c r="B47" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="C47" s="4" t="s">
+      <c r="C47" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="D47" s="4" t="s">
+      <c r="D47" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="50.4" x14ac:dyDescent="0.3">
-      <c r="A48" s="4" t="s">
+      <c r="A48" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="B48" s="4" t="s">
+      <c r="B48" s="3" t="s">
         <v>231</v>
       </c>
-      <c r="C48" s="4" t="s">
+      <c r="C48" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="D48" s="4" t="s">
+      <c r="D48" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A49" s="4" t="s">
+      <c r="A49" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="B49" s="5" t="s">
+      <c r="B49" s="4" t="s">
         <v>253</v>
       </c>
-      <c r="C49" s="4" t="s">
+      <c r="C49" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="D49" s="4" t="s">
+      <c r="D49" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A50" s="4" t="s">
+      <c r="A50" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="B50" s="5" t="s">
+      <c r="B50" s="4" t="s">
         <v>252</v>
       </c>
-      <c r="C50" s="4" t="s">
+      <c r="C50" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="D50" s="4" t="s">
+      <c r="D50" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A51" s="4" t="s">
+      <c r="A51" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="B51" s="4" t="s">
+      <c r="B51" s="3" t="s">
         <v>234</v>
       </c>
-      <c r="C51" s="4" t="s">
+      <c r="C51" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="D51" s="4" t="s">
+      <c r="D51" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A52" s="4" t="s">
+      <c r="A52" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="B52" s="4" t="s">
+      <c r="B52" s="3" t="s">
         <v>235</v>
       </c>
-      <c r="C52" s="4" t="s">
+      <c r="C52" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="D52" s="4" t="s">
+      <c r="D52" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A53" s="4" t="s">
+      <c r="A53" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="B53" s="4" t="s">
+      <c r="B53" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="C53" s="4" t="s">
+      <c r="C53" s="3" t="s">
         <v>237</v>
       </c>
-      <c r="D53" s="4" t="s">
+      <c r="D53" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A54" s="4" t="s">
+      <c r="A54" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="B54" s="4" t="s">
+      <c r="B54" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="C54" s="4" t="s">
+      <c r="C54" s="3" t="s">
         <v>239</v>
       </c>
-      <c r="D54" s="4" t="s">
+      <c r="D54" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A55" s="4" t="s">
+      <c r="A55" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="B55" s="4" t="s">
+      <c r="B55" s="3" t="s">
         <v>240</v>
       </c>
-      <c r="C55" s="4" t="s">
+      <c r="C55" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="D55" s="4" t="s">
+      <c r="D55" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A56" s="4" t="s">
+      <c r="A56" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="B56" s="4" t="s">
+      <c r="B56" s="3" t="s">
         <v>241</v>
       </c>
-      <c r="C56" s="4" t="s">
+      <c r="C56" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="D56" s="4" t="s">
+      <c r="D56" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A57" s="4" t="s">
+      <c r="A57" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="B57" s="4" t="s">
+      <c r="B57" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="C57" s="4" t="s">
+      <c r="C57" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="D57" s="4" t="s">
+      <c r="D57" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A58" s="4" t="s">
+      <c r="A58" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="B58" s="4" t="s">
+      <c r="B58" s="3" t="s">
         <v>243</v>
       </c>
-      <c r="C58" s="4" t="s">
+      <c r="C58" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="D58" s="4" t="s">
+      <c r="D58" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A59" s="4" t="s">
+      <c r="A59" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="B59" s="4" t="s">
+      <c r="B59" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="C59" s="4" t="s">
+      <c r="C59" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="D59" s="4" t="s">
+      <c r="D59" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A60" s="4" t="s">
+      <c r="A60" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="B60" s="4" t="s">
+      <c r="B60" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="C60" s="4" t="s">
+      <c r="C60" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="D60" s="4" t="s">
+      <c r="D60" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A61" s="4" t="s">
+      <c r="A61" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="B61" s="4" t="s">
+      <c r="B61" s="3" t="s">
         <v>246</v>
       </c>
-      <c r="C61" s="4" t="s">
+      <c r="C61" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="D61" s="4" t="s">
+      <c r="D61" s="3" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A62" s="4" t="s">
+      <c r="A62" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="B62" s="4" t="s">
+      <c r="B62" s="3" t="s">
         <v>247</v>
       </c>
-      <c r="C62" s="4" t="s">
+      <c r="C62" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="D62" s="4" t="s">
+      <c r="D62" s="3" t="s">
         <v>251</v>
       </c>
     </row>

</xml_diff>